<commit_message>
chore: publish xdsdocuments IG 1.0.0-trial-use-2
</commit_message>
<xml_diff>
--- a/ig/xdsdocuments/StructureDefinition-homecare-observation-documentreference.xlsx
+++ b/ig/xdsdocuments/StructureDefinition-homecare-observation-documentreference.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0-trial-use-1</t>
+    <t>1.0.0-trial-use-2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-01T09:36:40+00:00</t>
+    <t>2026-06-17T08:46:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -759,7 +759,7 @@
     <t>While each resource, including the DocumentReference itself, has its own version identifier, this is a formal identifier for the logical version of the DocumentReference as a whole. It would remain constant if the resources were moved to a new server, and all got new individual resource versions, for example.</t>
   </si>
   <si>
-    <t>1.0-trial-use-1</t>
+    <t>2.0</t>
   </si>
   <si>
     <t>Extension.value[x]</t>

</xml_diff>

<commit_message>
chore: publish xdsdocuments IG 1.0.0-trial-use-2 (#85)
Co-authored-by: tmsMedcom <tmsMedcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/xdsdocuments/StructureDefinition-homecare-observation-documentreference.xlsx
+++ b/ig/xdsdocuments/StructureDefinition-homecare-observation-documentreference.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0-trial-use-1</t>
+    <t>1.0.0-trial-use-2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-01T09:36:40+00:00</t>
+    <t>2026-06-17T08:46:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -759,7 +759,7 @@
     <t>While each resource, including the DocumentReference itself, has its own version identifier, this is a formal identifier for the logical version of the DocumentReference as a whole. It would remain constant if the resources were moved to a new server, and all got new individual resource versions, for example.</t>
   </si>
   <si>
-    <t>1.0-trial-use-1</t>
+    <t>2.0</t>
   </si>
   <si>
     <t>Extension.value[x]</t>

</xml_diff>